<commit_message>
fix(linzess): SEO for savings-card terms page (h1 + meta description)
PageSpeed SEO/a11y flagged the terms page for no meta description and a
missing top-level <h1> (lead heading was an <h2>). Build the terms page
deterministically in a new transformer (verbatim regulated copy + <h1> +
terms-content section + curated brand/title/description metadata) instead
of trusting the unreliable live scrape, and write it to the correct
/linzess/savings-card/terms path.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-savings-card-subpage.report.xlsx
+++ b/tools/importer/reports/import-savings-card-subpage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="46">
   <si>
     <t>_reportFile</t>
   </si>
@@ -82,13 +82,73 @@
     <t>savings-card/terms</t>
   </si>
   <si>
-    <t>2026-06-05T06:49:16.045Z</t>
+    <t>2026-06-19T10:37:46.341Z</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
     <t>https://www.linzess.com/savings-card/terms</t>
+  </si>
+  <si>
+    <t>linzess/savings-card/terms.report.json</t>
+  </si>
+  <si>
+    <t>linzess/savings-card/terms</t>
+  </si>
+  <si>
+    <t>2026-06-19T10:41:01.005Z</t>
+  </si>
+  <si>
+    <t>linzess/utility/es-home.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards-grid","columns","accordion","text-container"]</t>
+  </si>
+  <si>
+    <t>linzess/utility/es-home</t>
+  </si>
+  <si>
+    <t>linzess-es-home</t>
+  </si>
+  <si>
+    <t>2026-06-14T16:30:15.126Z</t>
+  </si>
+  <si>
+    <t>ES LINZESS homepage</t>
+  </si>
+  <si>
+    <t>https://es.linzess.com/</t>
+  </si>
+  <si>
+    <t>linzess/utility/reminder-terms-conditions.report.json</t>
+  </si>
+  <si>
+    <t>linzess/utility/reminder-terms-conditions</t>
+  </si>
+  <si>
+    <t>linzess-utility</t>
+  </si>
+  <si>
+    <t>2026-06-15T06:17:58.992Z</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/reminder-terms-conditions</t>
+  </si>
+  <si>
+    <t>linzess/utility/sitemap.report.json</t>
+  </si>
+  <si>
+    <t>linzess/utility/sitemap</t>
+  </si>
+  <si>
+    <t>2026-06-19T08:36:13.870Z</t>
+  </si>
+  <si>
+    <t>Sitemap | LINZESS® (linaclotide)</t>
+  </si>
+  <si>
+    <t>https://www.linzess.com/sitemap</t>
   </si>
 </sst>
 </file>
@@ -477,16 +537,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="43" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="43" customWidth="1"/>
-    <col min="8" max="8" width="47" customWidth="1"/>
+    <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -591,6 +650,110 @@
       </c>
       <c r="H4" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>